<commit_message>
Rebalance RH134 teaching to 3 chapters/week
Move week 7's row from the RH134 table into the RH124 table where it
belongs (Weeks 1 to 7). Regroup RH134 chapters more evenly across
weeks 8-13:

- Week 9: chapters 4-6 (was 4-5) — SELinux moves in
- Week 10: chapters 7-9 (was 6-9) — SELinux moves out
- Week 12: chapters 13-15 (was 13-16) — installation moves out
- Week 13: chapters 16-18 (was 17-18) — installation moves in

Weeks 8 and 11 are unchanged; revision stays week 14 and the exam
stays week 15.

Update objective mapping weeks in coverage.md, the challenge 14
readiness week in practice.md, weekly reading sections and
cross-references in readings.md, planner/build.py's WEEKS/NOTES/
PRACTICE data (and rebuild the generated spreadsheet), and a stale
"twelve weeks... catch-up" description of lessons.md in README.md.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/planner/ict257-study-planner.xlsx
+++ b/planner/ict257-study-planner.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Start here" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Study plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Practice" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Practice" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="SemesterStart">'Start here'!$B$5</definedName>
@@ -1003,14 +1003,14 @@
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>Weeks 1 to 6 are RH124. Weeks 7 to 12 are RH134. Week 13 is catch-up, week 14 is revision, and you sit the exam in week 15.</t>
+          <t>Weeks 1 to 7 are RH124. Weeks 8 to 13 are RH134. Week 14 is revision, and you sit the exam in week 15.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>The two comprehensive reviews sit in weeks 13 and 14, where lessons.md puts them. RH124 20 is open to you from week 6 and RH134 19.02 to 19.04 from week 11, so start either one early if you can.</t>
+          <t>The two comprehensive reviews sit in week 14, where lessons.md puts them. RH124 20 is open to you from week 7 and RH134 19.02 to 19.04 from week 12, so start either one early if you can.</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>Three weeks after the first revision falls past the exam for the week 11 and week 12 chapters. Those second revisions are pulled back into revision week instead, week 11 material first and week 12 material a day later.</t>
+          <t>Three weeks after the first revision falls past the exam for the week 12 and week 13 chapters. Those second revisions are pulled back into revision week instead, week 12 material first and week 13 material a day later.</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
         <v/>
       </c>
       <c r="H5" s="22">
-        <f>IF(OR($B5=0,$D5&gt;=13),"",MIN($G5+21,RevisionCutoff-12+$D5))</f>
+        <f>IF(OR($B5=0,$D5&gt;=14),"",MIN($G5+21,RevisionCutoff-13+$D5))</f>
         <v/>
       </c>
       <c r="I5" s="23" t="inlineStr">
@@ -1271,7 +1271,7 @@
         <v/>
       </c>
       <c r="H6" s="22">
-        <f>IF(OR($B6=0,$D6&gt;=13),"",MIN($G6+21,RevisionCutoff-12+$D6))</f>
+        <f>IF(OR($B6=0,$D6&gt;=14),"",MIN($G6+21,RevisionCutoff-13+$D6))</f>
         <v/>
       </c>
       <c r="I6" s="23" t="inlineStr">
@@ -1317,7 +1317,7 @@
         <v/>
       </c>
       <c r="H7" s="22">
-        <f>IF(OR($B7=0,$D7&gt;=13),"",MIN($G7+21,RevisionCutoff-12+$D7))</f>
+        <f>IF(OR($B7=0,$D7&gt;=14),"",MIN($G7+21,RevisionCutoff-13+$D7))</f>
         <v/>
       </c>
       <c r="I7" s="23" t="inlineStr">
@@ -1359,7 +1359,7 @@
         <v/>
       </c>
       <c r="H8" s="22">
-        <f>IF(OR($B8=0,$D8&gt;=13),"",MIN($G8+21,RevisionCutoff-12+$D8))</f>
+        <f>IF(OR($B8=0,$D8&gt;=14),"",MIN($G8+21,RevisionCutoff-13+$D8))</f>
         <v/>
       </c>
       <c r="I8" s="23" t="inlineStr">
@@ -1401,7 +1401,7 @@
         <v/>
       </c>
       <c r="H9" s="22">
-        <f>IF(OR($B9=0,$D9&gt;=13),"",MIN($G9+21,RevisionCutoff-12+$D9))</f>
+        <f>IF(OR($B9=0,$D9&gt;=14),"",MIN($G9+21,RevisionCutoff-13+$D9))</f>
         <v/>
       </c>
       <c r="I9" s="23" t="inlineStr">
@@ -1443,7 +1443,7 @@
         <v/>
       </c>
       <c r="H10" s="22">
-        <f>IF(OR($B10=0,$D10&gt;=13),"",MIN($G10+21,RevisionCutoff-12+$D10))</f>
+        <f>IF(OR($B10=0,$D10&gt;=14),"",MIN($G10+21,RevisionCutoff-13+$D10))</f>
         <v/>
       </c>
       <c r="I10" s="23" t="inlineStr">
@@ -1489,7 +1489,7 @@
         <v/>
       </c>
       <c r="H11" s="22">
-        <f>IF(OR($B11=0,$D11&gt;=13),"",MIN($G11+21,RevisionCutoff-12+$D11))</f>
+        <f>IF(OR($B11=0,$D11&gt;=14),"",MIN($G11+21,RevisionCutoff-13+$D11))</f>
         <v/>
       </c>
       <c r="I11" s="23" t="inlineStr">
@@ -1531,7 +1531,7 @@
         <v/>
       </c>
       <c r="H12" s="22">
-        <f>IF(OR($B12=0,$D12&gt;=13),"",MIN($G12+21,RevisionCutoff-12+$D12))</f>
+        <f>IF(OR($B12=0,$D12&gt;=14),"",MIN($G12+21,RevisionCutoff-13+$D12))</f>
         <v/>
       </c>
       <c r="I12" s="23" t="inlineStr">
@@ -1573,7 +1573,7 @@
         <v/>
       </c>
       <c r="H13" s="22">
-        <f>IF(OR($B13=0,$D13&gt;=13),"",MIN($G13+21,RevisionCutoff-12+$D13))</f>
+        <f>IF(OR($B13=0,$D13&gt;=14),"",MIN($G13+21,RevisionCutoff-13+$D13))</f>
         <v/>
       </c>
       <c r="I13" s="23" t="inlineStr">
@@ -1615,7 +1615,7 @@
         <v/>
       </c>
       <c r="H14" s="22">
-        <f>IF(OR($B14=0,$D14&gt;=13),"",MIN($G14+21,RevisionCutoff-12+$D14))</f>
+        <f>IF(OR($B14=0,$D14&gt;=14),"",MIN($G14+21,RevisionCutoff-13+$D14))</f>
         <v/>
       </c>
       <c r="I14" s="23" t="inlineStr">
@@ -1657,7 +1657,7 @@
         <v/>
       </c>
       <c r="H15" s="22">
-        <f>IF(OR($B15=0,$D15&gt;=13),"",MIN($G15+21,RevisionCutoff-12+$D15))</f>
+        <f>IF(OR($B15=0,$D15&gt;=14),"",MIN($G15+21,RevisionCutoff-13+$D15))</f>
         <v/>
       </c>
       <c r="I15" s="23" t="inlineStr">
@@ -1699,7 +1699,7 @@
         <v/>
       </c>
       <c r="H16" s="22">
-        <f>IF(OR($B16=0,$D16&gt;=13),"",MIN($G16+21,RevisionCutoff-12+$D16))</f>
+        <f>IF(OR($B16=0,$D16&gt;=14),"",MIN($G16+21,RevisionCutoff-13+$D16))</f>
         <v/>
       </c>
       <c r="I16" s="23" t="inlineStr">
@@ -1725,11 +1725,11 @@
         </is>
       </c>
       <c r="D17" s="19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E17" s="21" t="inlineStr">
         <is>
-          <t>File permissions, RPM packages and Flatpak applications</t>
+          <t>Software repositories, Flatpak applications and removable media</t>
         </is>
       </c>
       <c r="F17" s="22">
@@ -1741,7 +1741,7 @@
         <v/>
       </c>
       <c r="H17" s="22">
-        <f>IF(OR($B17=0,$D17&gt;=13),"",MIN($G17+21,RevisionCutoff-12+$D17))</f>
+        <f>IF(OR($B17=0,$D17&gt;=14),"",MIN($G17+21,RevisionCutoff-13+$D17))</f>
         <v/>
       </c>
       <c r="I17" s="23" t="inlineStr">
@@ -1767,11 +1767,11 @@
         </is>
       </c>
       <c r="D18" s="19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E18" s="21" t="inlineStr">
         <is>
-          <t>File permissions, RPM packages and Flatpak applications</t>
+          <t>Software repositories, Flatpak applications and removable media</t>
         </is>
       </c>
       <c r="F18" s="22">
@@ -1783,7 +1783,7 @@
         <v/>
       </c>
       <c r="H18" s="22">
-        <f>IF(OR($B18=0,$D18&gt;=13),"",MIN($G18+21,RevisionCutoff-12+$D18))</f>
+        <f>IF(OR($B18=0,$D18&gt;=14),"",MIN($G18+21,RevisionCutoff-13+$D18))</f>
         <v/>
       </c>
       <c r="I18" s="23" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="E19" s="21" t="inlineStr">
         <is>
-          <t>File systems, locating files, processes and system services</t>
+          <t>Software repositories, Flatpak applications and removable media</t>
         </is>
       </c>
       <c r="F19" s="22">
@@ -1825,7 +1825,7 @@
         <v/>
       </c>
       <c r="H19" s="22">
-        <f>IF(OR($B19=0,$D19&gt;=13),"",MIN($G19+21,RevisionCutoff-12+$D19))</f>
+        <f>IF(OR($B19=0,$D19&gt;=14),"",MIN($G19+21,RevisionCutoff-13+$D19))</f>
         <v/>
       </c>
       <c r="I19" s="23" t="inlineStr">
@@ -1851,11 +1851,11 @@
         </is>
       </c>
       <c r="D20" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E20" s="21" t="inlineStr">
         <is>
-          <t>File systems, locating files, processes and system services</t>
+          <t>Processes, system services and remote access</t>
         </is>
       </c>
       <c r="F20" s="22">
@@ -1867,7 +1867,7 @@
         <v/>
       </c>
       <c r="H20" s="22">
-        <f>IF(OR($B20=0,$D20&gt;=13),"",MIN($G20+21,RevisionCutoff-12+$D20))</f>
+        <f>IF(OR($B20=0,$D20&gt;=14),"",MIN($G20+21,RevisionCutoff-13+$D20))</f>
         <v/>
       </c>
       <c r="I20" s="23" t="inlineStr">
@@ -1893,11 +1893,11 @@
         </is>
       </c>
       <c r="D21" s="19" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" s="21" t="inlineStr">
         <is>
-          <t>File systems, locating files, processes and system services</t>
+          <t>Processes, system services and remote access</t>
         </is>
       </c>
       <c r="F21" s="22">
@@ -1909,7 +1909,7 @@
         <v/>
       </c>
       <c r="H21" s="22">
-        <f>IF(OR($B21=0,$D21&gt;=13),"",MIN($G21+21,RevisionCutoff-12+$D21))</f>
+        <f>IF(OR($B21=0,$D21&gt;=14),"",MIN($G21+21,RevisionCutoff-13+$D21))</f>
         <v/>
       </c>
       <c r="I21" s="23" t="inlineStr">
@@ -1935,11 +1935,11 @@
         </is>
       </c>
       <c r="D22" s="19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E22" s="21" t="inlineStr">
         <is>
-          <t>Network addressing and configuration, name resolution and secure remote access</t>
+          <t>Network configuration, name resolution and secure remote access</t>
         </is>
       </c>
       <c r="F22" s="22">
@@ -1951,7 +1951,7 @@
         <v/>
       </c>
       <c r="H22" s="22">
-        <f>IF(OR($B22=0,$D22&gt;=13),"",MIN($G22+21,RevisionCutoff-12+$D22))</f>
+        <f>IF(OR($B22=0,$D22&gt;=14),"",MIN($G22+21,RevisionCutoff-13+$D22))</f>
         <v/>
       </c>
       <c r="I22" s="23" t="inlineStr">
@@ -1977,11 +1977,11 @@
         </is>
       </c>
       <c r="D23" s="19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E23" s="21" t="inlineStr">
         <is>
-          <t>Network addressing and configuration, name resolution and secure remote access</t>
+          <t>Network configuration, name resolution and secure remote access</t>
         </is>
       </c>
       <c r="F23" s="22">
@@ -1993,7 +1993,7 @@
         <v/>
       </c>
       <c r="H23" s="22">
-        <f>IF(OR($B23=0,$D23&gt;=13),"",MIN($G23+21,RevisionCutoff-12+$D23))</f>
+        <f>IF(OR($B23=0,$D23&gt;=14),"",MIN($G23+21,RevisionCutoff-13+$D23))</f>
         <v/>
       </c>
       <c r="I23" s="23" t="inlineStr">
@@ -2019,11 +2019,11 @@
         </is>
       </c>
       <c r="D24" s="19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E24" s="21" t="inlineStr">
         <is>
-          <t>Network addressing and configuration, name resolution and secure remote access</t>
+          <t>Network configuration, name resolution and secure remote access</t>
         </is>
       </c>
       <c r="F24" s="22">
@@ -2035,7 +2035,7 @@
         <v/>
       </c>
       <c r="H24" s="22">
-        <f>IF(OR($B24=0,$D24&gt;=13),"",MIN($G24+21,RevisionCutoff-12+$D24))</f>
+        <f>IF(OR($B24=0,$D24&gt;=14),"",MIN($G24+21,RevisionCutoff-13+$D24))</f>
         <v/>
       </c>
       <c r="I24" s="23" t="inlineStr">
@@ -2061,11 +2061,11 @@
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E25" s="21" t="inlineStr">
         <is>
-          <t>Catch-up week. No new chapters. Overflow from the twelve teaching weeks.</t>
+          <t>Revision week. Objective by objective, with both comprehensive reviews open to you.</t>
         </is>
       </c>
       <c r="F25" s="22">
@@ -2077,7 +2077,7 @@
         <v/>
       </c>
       <c r="H25" s="22">
-        <f>IF(OR($B25=0,$D25&gt;=13),"",MIN($G25+21,RevisionCutoff-12+$D25))</f>
+        <f>IF(OR($B25=0,$D25&gt;=14),"",MIN($G25+21,RevisionCutoff-13+$D25))</f>
         <v/>
       </c>
       <c r="I25" s="23" t="inlineStr">
@@ -2088,7 +2088,7 @@
       <c r="J25" s="23" t="n"/>
       <c r="K25" s="21" t="inlineStr">
         <is>
-          <t>Five review labs. Open to you from week 6, so start earlier if you can.</t>
+          <t>Five review labs. Open to you from week 7, so start earlier if you can.</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="E26" s="27" t="inlineStr">
         <is>
-          <t>Shell scripts, regular expressions and scheduled jobs</t>
+          <t>Network configuration, name resolution and secure remote access</t>
         </is>
       </c>
       <c r="F26" s="28">
@@ -2123,7 +2123,7 @@
         <v/>
       </c>
       <c r="H26" s="28">
-        <f>IF(OR($B26=0,$D26&gt;=13),"",MIN($G26+21,RevisionCutoff-12+$D26))</f>
+        <f>IF(OR($B26=0,$D26&gt;=14),"",MIN($G26+21,RevisionCutoff-13+$D26))</f>
         <v/>
       </c>
       <c r="I26" s="29" t="inlineStr">
@@ -2153,11 +2153,11 @@
         </is>
       </c>
       <c r="D27" s="19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E27" s="21" t="inlineStr">
         <is>
-          <t>Shell scripts, regular expressions and scheduled jobs</t>
+          <t>Shell scripts, regular expressions and scheduled user tasks</t>
         </is>
       </c>
       <c r="F27" s="22">
@@ -2169,7 +2169,7 @@
         <v/>
       </c>
       <c r="H27" s="22">
-        <f>IF(OR($B27=0,$D27&gt;=13),"",MIN($G27+21,RevisionCutoff-12+$D27))</f>
+        <f>IF(OR($B27=0,$D27&gt;=14),"",MIN($G27+21,RevisionCutoff-13+$D27))</f>
         <v/>
       </c>
       <c r="I27" s="23" t="inlineStr">
@@ -2195,11 +2195,11 @@
         </is>
       </c>
       <c r="D28" s="19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E28" s="21" t="inlineStr">
         <is>
-          <t>Shell scripts, regular expressions and scheduled jobs</t>
+          <t>Shell scripts, regular expressions and scheduled user tasks</t>
         </is>
       </c>
       <c r="F28" s="22">
@@ -2211,7 +2211,7 @@
         <v/>
       </c>
       <c r="H28" s="22">
-        <f>IF(OR($B28=0,$D28&gt;=13),"",MIN($G28+21,RevisionCutoff-12+$D28))</f>
+        <f>IF(OR($B28=0,$D28&gt;=14),"",MIN($G28+21,RevisionCutoff-13+$D28))</f>
         <v/>
       </c>
       <c r="I28" s="23" t="inlineStr">
@@ -2237,11 +2237,11 @@
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E29" s="21" t="inlineStr">
         <is>
-          <t>Shell scripts, regular expressions and scheduled jobs</t>
+          <t>Shell scripts, regular expressions and scheduled user tasks</t>
         </is>
       </c>
       <c r="F29" s="22">
@@ -2253,7 +2253,7 @@
         <v/>
       </c>
       <c r="H29" s="22">
-        <f>IF(OR($B29=0,$D29&gt;=13),"",MIN($G29+21,RevisionCutoff-12+$D29))</f>
+        <f>IF(OR($B29=0,$D29&gt;=14),"",MIN($G29+21,RevisionCutoff-13+$D29))</f>
         <v/>
       </c>
       <c r="I29" s="23" t="inlineStr">
@@ -2279,11 +2279,11 @@
         </is>
       </c>
       <c r="D30" s="19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E30" s="21" t="inlineStr">
         <is>
-          <t>Recurring jobs, logs, journals and keeping time</t>
+          <t>Recurring system tasks, logs, journals, keeping time and SELinux</t>
         </is>
       </c>
       <c r="F30" s="22">
@@ -2295,7 +2295,7 @@
         <v/>
       </c>
       <c r="H30" s="22">
-        <f>IF(OR($B30=0,$D30&gt;=13),"",MIN($G30+21,RevisionCutoff-12+$D30))</f>
+        <f>IF(OR($B30=0,$D30&gt;=14),"",MIN($G30+21,RevisionCutoff-13+$D30))</f>
         <v/>
       </c>
       <c r="I30" s="23" t="inlineStr">
@@ -2321,11 +2321,11 @@
         </is>
       </c>
       <c r="D31" s="19" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E31" s="21" t="inlineStr">
         <is>
-          <t>Recurring jobs, logs, journals and keeping time</t>
+          <t>Recurring system tasks, logs, journals, keeping time and SELinux</t>
         </is>
       </c>
       <c r="F31" s="22">
@@ -2337,7 +2337,7 @@
         <v/>
       </c>
       <c r="H31" s="22">
-        <f>IF(OR($B31=0,$D31&gt;=13),"",MIN($G31+21,RevisionCutoff-12+$D31))</f>
+        <f>IF(OR($B31=0,$D31&gt;=14),"",MIN($G31+21,RevisionCutoff-13+$D31))</f>
         <v/>
       </c>
       <c r="I31" s="23" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="E32" s="21" t="inlineStr">
         <is>
-          <t>SELinux, archives, secure file transfer and tuning profiles</t>
+          <t>Recurring system tasks, logs, journals, keeping time and SELinux</t>
         </is>
       </c>
       <c r="F32" s="22">
@@ -2379,7 +2379,7 @@
         <v/>
       </c>
       <c r="H32" s="22">
-        <f>IF(OR($B32=0,$D32&gt;=13),"",MIN($G32+21,RevisionCutoff-12+$D32))</f>
+        <f>IF(OR($B32=0,$D32&gt;=14),"",MIN($G32+21,RevisionCutoff-13+$D32))</f>
         <v/>
       </c>
       <c r="I32" s="23" t="inlineStr">
@@ -2390,7 +2390,7 @@
       <c r="J32" s="23" t="n"/>
       <c r="K32" s="21" t="inlineStr">
         <is>
-          <t>Hardest third of the module starts here. Weeks 9 to 11 deserve the most revision time.</t>
+          <t>Hardest third of the module starts here. Weeks 9, 11 and 12 deserve the most revision time.</t>
         </is>
       </c>
     </row>
@@ -2409,11 +2409,11 @@
         </is>
       </c>
       <c r="D33" s="19" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E33" s="21" t="inlineStr">
         <is>
-          <t>SELinux, archives, secure file transfer and tuning profiles</t>
+          <t>Archives, secure file transfer and tuning profiles</t>
         </is>
       </c>
       <c r="F33" s="22">
@@ -2425,7 +2425,7 @@
         <v/>
       </c>
       <c r="H33" s="22">
-        <f>IF(OR($B33=0,$D33&gt;=13),"",MIN($G33+21,RevisionCutoff-12+$D33))</f>
+        <f>IF(OR($B33=0,$D33&gt;=14),"",MIN($G33+21,RevisionCutoff-13+$D33))</f>
         <v/>
       </c>
       <c r="I33" s="23" t="inlineStr">
@@ -2451,11 +2451,11 @@
         </is>
       </c>
       <c r="D34" s="19" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E34" s="21" t="inlineStr">
         <is>
-          <t>SELinux, archives, secure file transfer and tuning profiles</t>
+          <t>Archives, secure file transfer and tuning profiles</t>
         </is>
       </c>
       <c r="F34" s="22">
@@ -2467,7 +2467,7 @@
         <v/>
       </c>
       <c r="H34" s="22">
-        <f>IF(OR($B34=0,$D34&gt;=13),"",MIN($G34+21,RevisionCutoff-12+$D34))</f>
+        <f>IF(OR($B34=0,$D34&gt;=14),"",MIN($G34+21,RevisionCutoff-13+$D34))</f>
         <v/>
       </c>
       <c r="I34" s="23" t="inlineStr">
@@ -2493,11 +2493,11 @@
         </is>
       </c>
       <c r="D35" s="19" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E35" s="21" t="inlineStr">
         <is>
-          <t>SELinux, archives, secure file transfer and tuning profiles</t>
+          <t>Archives, secure file transfer and tuning profiles</t>
         </is>
       </c>
       <c r="F35" s="22">
@@ -2509,7 +2509,7 @@
         <v/>
       </c>
       <c r="H35" s="22">
-        <f>IF(OR($B35=0,$D35&gt;=13),"",MIN($G35+21,RevisionCutoff-12+$D35))</f>
+        <f>IF(OR($B35=0,$D35&gt;=14),"",MIN($G35+21,RevisionCutoff-13+$D35))</f>
         <v/>
       </c>
       <c r="I35" s="23" t="inlineStr">
@@ -2535,7 +2535,7 @@
         </is>
       </c>
       <c r="D36" s="19" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E36" s="21" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
         <v/>
       </c>
       <c r="H36" s="22">
-        <f>IF(OR($B36=0,$D36&gt;=13),"",MIN($G36+21,RevisionCutoff-12+$D36))</f>
+        <f>IF(OR($B36=0,$D36&gt;=14),"",MIN($G36+21,RevisionCutoff-13+$D36))</f>
         <v/>
       </c>
       <c r="I36" s="23" t="inlineStr">
@@ -2577,7 +2577,7 @@
         </is>
       </c>
       <c r="D37" s="19" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E37" s="21" t="inlineStr">
         <is>
@@ -2593,7 +2593,7 @@
         <v/>
       </c>
       <c r="H37" s="22">
-        <f>IF(OR($B37=0,$D37&gt;=13),"",MIN($G37+21,RevisionCutoff-12+$D37))</f>
+        <f>IF(OR($B37=0,$D37&gt;=14),"",MIN($G37+21,RevisionCutoff-13+$D37))</f>
         <v/>
       </c>
       <c r="I37" s="23" t="inlineStr">
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="D38" s="19" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E38" s="21" t="inlineStr">
         <is>
@@ -2635,7 +2635,7 @@
         <v/>
       </c>
       <c r="H38" s="22">
-        <f>IF(OR($B38=0,$D38&gt;=13),"",MIN($G38+21,RevisionCutoff-12+$D38))</f>
+        <f>IF(OR($B38=0,$D38&gt;=14),"",MIN($G38+21,RevisionCutoff-13+$D38))</f>
         <v/>
       </c>
       <c r="I38" s="23" t="inlineStr">
@@ -2661,11 +2661,11 @@
         </is>
       </c>
       <c r="D39" s="19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E39" s="21" t="inlineStr">
         <is>
-          <t>Boot troubleshooting, firewalls, network file systems and installation</t>
+          <t>Boot troubleshooting, firewalls and network file systems</t>
         </is>
       </c>
       <c r="F39" s="22">
@@ -2677,7 +2677,7 @@
         <v/>
       </c>
       <c r="H39" s="22">
-        <f>IF(OR($B39=0,$D39&gt;=13),"",MIN($G39+21,RevisionCutoff-12+$D39))</f>
+        <f>IF(OR($B39=0,$D39&gt;=14),"",MIN($G39+21,RevisionCutoff-13+$D39))</f>
         <v/>
       </c>
       <c r="I39" s="23" t="inlineStr">
@@ -2703,11 +2703,11 @@
         </is>
       </c>
       <c r="D40" s="19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E40" s="21" t="inlineStr">
         <is>
-          <t>Boot troubleshooting, firewalls, network file systems and installation</t>
+          <t>Boot troubleshooting, firewalls and network file systems</t>
         </is>
       </c>
       <c r="F40" s="22">
@@ -2719,7 +2719,7 @@
         <v/>
       </c>
       <c r="H40" s="22">
-        <f>IF(OR($B40=0,$D40&gt;=13),"",MIN($G40+21,RevisionCutoff-12+$D40))</f>
+        <f>IF(OR($B40=0,$D40&gt;=14),"",MIN($G40+21,RevisionCutoff-13+$D40))</f>
         <v/>
       </c>
       <c r="I40" s="23" t="inlineStr">
@@ -2745,11 +2745,11 @@
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E41" s="21" t="inlineStr">
         <is>
-          <t>Boot troubleshooting, firewalls, network file systems and installation</t>
+          <t>Boot troubleshooting, firewalls and network file systems</t>
         </is>
       </c>
       <c r="F41" s="22">
@@ -2761,7 +2761,7 @@
         <v/>
       </c>
       <c r="H41" s="22">
-        <f>IF(OR($B41=0,$D41&gt;=13),"",MIN($G41+21,RevisionCutoff-12+$D41))</f>
+        <f>IF(OR($B41=0,$D41&gt;=14),"",MIN($G41+21,RevisionCutoff-13+$D41))</f>
         <v/>
       </c>
       <c r="I41" s="23" t="inlineStr">
@@ -2787,11 +2787,11 @@
         </is>
       </c>
       <c r="D42" s="19" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E42" s="21" t="inlineStr">
         <is>
-          <t>Boot troubleshooting, firewalls, network file systems and installation</t>
+          <t>Installation, containers and image mode</t>
         </is>
       </c>
       <c r="F42" s="22">
@@ -2803,7 +2803,7 @@
         <v/>
       </c>
       <c r="H42" s="22">
-        <f>IF(OR($B42=0,$D42&gt;=13),"",MIN($G42+21,RevisionCutoff-12+$D42))</f>
+        <f>IF(OR($B42=0,$D42&gt;=14),"",MIN($G42+21,RevisionCutoff-13+$D42))</f>
         <v/>
       </c>
       <c r="I42" s="23" t="inlineStr">
@@ -2833,11 +2833,11 @@
         </is>
       </c>
       <c r="D43" s="19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E43" s="21" t="inlineStr">
         <is>
-          <t>Containers and image mode</t>
+          <t>Installation, containers and image mode</t>
         </is>
       </c>
       <c r="F43" s="22">
@@ -2849,7 +2849,7 @@
         <v/>
       </c>
       <c r="H43" s="22">
-        <f>IF(OR($B43=0,$D43&gt;=13),"",MIN($G43+21,RevisionCutoff-12+$D43))</f>
+        <f>IF(OR($B43=0,$D43&gt;=14),"",MIN($G43+21,RevisionCutoff-13+$D43))</f>
         <v/>
       </c>
       <c r="I43" s="23" t="inlineStr">
@@ -2879,11 +2879,11 @@
         </is>
       </c>
       <c r="D44" s="19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E44" s="21" t="inlineStr">
         <is>
-          <t>Containers and image mode</t>
+          <t>Installation, containers and image mode</t>
         </is>
       </c>
       <c r="F44" s="22">
@@ -2895,7 +2895,7 @@
         <v/>
       </c>
       <c r="H44" s="22">
-        <f>IF(OR($B44=0,$D44&gt;=13),"",MIN($G44+21,RevisionCutoff-12+$D44))</f>
+        <f>IF(OR($B44=0,$D44&gt;=14),"",MIN($G44+21,RevisionCutoff-13+$D44))</f>
         <v/>
       </c>
       <c r="I44" s="23" t="inlineStr">
@@ -2941,7 +2941,7 @@
         <v/>
       </c>
       <c r="H45" s="22">
-        <f>IF(OR($B45=0,$D45&gt;=13),"",MIN($G45+21,RevisionCutoff-12+$D45))</f>
+        <f>IF(OR($B45=0,$D45&gt;=14),"",MIN($G45+21,RevisionCutoff-13+$D45))</f>
         <v/>
       </c>
       <c r="I45" s="23" t="inlineStr">
@@ -2952,7 +2952,7 @@
       <c r="J45" s="23" t="n"/>
       <c r="K45" s="21" t="inlineStr">
         <is>
-          <t>Labs 19.02 to 19.04 are open from week 11. Lab 19.05 rests on week 12 containers.</t>
+          <t>Labs 19.02 to 19.04 are open from week 12. Lab 19.05 rests on week 13 containers.</t>
         </is>
       </c>
     </row>
@@ -3376,11 +3376,11 @@
       </c>
       <c r="C12" s="30" t="inlineStr">
         <is>
-          <t>week 6</t>
+          <t>week 7</t>
         </is>
       </c>
       <c r="D12" s="22">
-        <f>SemesterStart+7*(6-1)</f>
+        <f>SemesterStart+7*(7-1)</f>
         <v/>
       </c>
       <c r="E12" s="19" t="inlineStr">
@@ -3416,11 +3416,11 @@
       </c>
       <c r="C13" s="30" t="inlineStr">
         <is>
-          <t>week 7</t>
+          <t>week 8</t>
         </is>
       </c>
       <c r="D13" s="22">
-        <f>SemesterStart+7*(7-1)</f>
+        <f>SemesterStart+7*(8-1)</f>
         <v/>
       </c>
       <c r="E13" s="19" t="inlineStr">
@@ -3456,11 +3456,11 @@
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>week 7</t>
+          <t>week 8</t>
         </is>
       </c>
       <c r="D14" s="22">
-        <f>SemesterStart+7*(7-1)</f>
+        <f>SemesterStart+7*(8-1)</f>
         <v/>
       </c>
       <c r="E14" s="19" t="inlineStr">
@@ -3496,11 +3496,11 @@
       </c>
       <c r="C15" s="30" t="inlineStr">
         <is>
-          <t>week 8</t>
+          <t>week 9</t>
         </is>
       </c>
       <c r="D15" s="22">
-        <f>SemesterStart+7*(8-1)</f>
+        <f>SemesterStart+7*(9-1)</f>
         <v/>
       </c>
       <c r="E15" s="19" t="inlineStr">
@@ -3536,11 +3536,11 @@
       </c>
       <c r="C16" s="30" t="inlineStr">
         <is>
-          <t>week 8</t>
+          <t>week 9</t>
         </is>
       </c>
       <c r="D16" s="22">
-        <f>SemesterStart+7*(8-1)</f>
+        <f>SemesterStart+7*(9-1)</f>
         <v/>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -3576,11 +3576,11 @@
       </c>
       <c r="C17" s="30" t="inlineStr">
         <is>
-          <t>week 9</t>
+          <t>week 10</t>
         </is>
       </c>
       <c r="D17" s="22">
-        <f>SemesterStart+7*(9-1)</f>
+        <f>SemesterStart+7*(10-1)</f>
         <v/>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -3656,11 +3656,11 @@
       </c>
       <c r="C19" s="30" t="inlineStr">
         <is>
-          <t>week 10</t>
+          <t>week 11</t>
         </is>
       </c>
       <c r="D19" s="22">
-        <f>SemesterStart+7*(10-1)</f>
+        <f>SemesterStart+7*(11-1)</f>
         <v/>
       </c>
       <c r="E19" s="19" t="inlineStr">
@@ -3696,11 +3696,11 @@
       </c>
       <c r="C20" s="30" t="inlineStr">
         <is>
-          <t>week 10</t>
+          <t>week 11</t>
         </is>
       </c>
       <c r="D20" s="22">
-        <f>SemesterStart+7*(10-1)</f>
+        <f>SemesterStart+7*(11-1)</f>
         <v/>
       </c>
       <c r="E20" s="19" t="inlineStr">
@@ -3736,11 +3736,11 @@
       </c>
       <c r="C21" s="30" t="inlineStr">
         <is>
-          <t>week 10</t>
+          <t>week 11</t>
         </is>
       </c>
       <c r="D21" s="22">
-        <f>SemesterStart+7*(10-1)</f>
+        <f>SemesterStart+7*(11-1)</f>
         <v/>
       </c>
       <c r="E21" s="19" t="inlineStr">
@@ -3776,11 +3776,11 @@
       </c>
       <c r="C22" s="30" t="inlineStr">
         <is>
-          <t>week 11</t>
+          <t>week 12</t>
         </is>
       </c>
       <c r="D22" s="22">
-        <f>SemesterStart+7*(11-1)</f>
+        <f>SemesterStart+7*(12-1)</f>
         <v/>
       </c>
       <c r="E22" s="19" t="inlineStr">
@@ -3816,11 +3816,11 @@
       </c>
       <c r="C23" s="30" t="inlineStr">
         <is>
-          <t>week 11</t>
+          <t>week 12</t>
         </is>
       </c>
       <c r="D23" s="22">
-        <f>SemesterStart+7*(11-1)</f>
+        <f>SemesterStart+7*(12-1)</f>
         <v/>
       </c>
       <c r="E23" s="19" t="inlineStr">
@@ -3856,11 +3856,11 @@
       </c>
       <c r="C24" s="30" t="inlineStr">
         <is>
-          <t>week 11</t>
+          <t>week 12</t>
         </is>
       </c>
       <c r="D24" s="22">
-        <f>SemesterStart+7*(11-1)</f>
+        <f>SemesterStart+7*(12-1)</f>
         <v/>
       </c>
       <c r="E24" s="19" t="inlineStr">
@@ -3896,11 +3896,11 @@
       </c>
       <c r="C25" s="30" t="inlineStr">
         <is>
-          <t>week 11</t>
+          <t>week 12</t>
         </is>
       </c>
       <c r="D25" s="22">
-        <f>SemesterStart+7*(11-1)</f>
+        <f>SemesterStart+7*(12-1)</f>
         <v/>
       </c>
       <c r="E25" s="19" t="inlineStr">
@@ -3936,11 +3936,11 @@
       </c>
       <c r="C26" s="30" t="inlineStr">
         <is>
-          <t>week 11</t>
+          <t>week 12</t>
         </is>
       </c>
       <c r="D26" s="22">
-        <f>SemesterStart+7*(11-1)</f>
+        <f>SemesterStart+7*(12-1)</f>
         <v/>
       </c>
       <c r="E26" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Move RH134 chapter 6 from week 9 to week 10
Week 9 ran out of time for SELinux. The chapter 6 sections, their
objectives (RHCSA-10.4 to 10.8), the coloring book reading and the
selinux-booleans practice challenge all follow, and the study
planner is rebuilt to match.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planner/ict257-study-planner.xlsx
+++ b/planner/ict257-study-planner.xlsx
@@ -2283,7 +2283,7 @@
       </c>
       <c r="E30" s="21" t="inlineStr">
         <is>
-          <t>Recurring system tasks, logs, journals, keeping time and SELinux</t>
+          <t>Recurring system tasks, logs, journals and keeping time</t>
         </is>
       </c>
       <c r="F30" s="22">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="E31" s="21" t="inlineStr">
         <is>
-          <t>Recurring system tasks, logs, journals, keeping time and SELinux</t>
+          <t>Recurring system tasks, logs, journals and keeping time</t>
         </is>
       </c>
       <c r="F31" s="22">
@@ -2363,11 +2363,11 @@
         </is>
       </c>
       <c r="D32" s="19" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E32" s="21" t="inlineStr">
         <is>
-          <t>Recurring system tasks, logs, journals, keeping time and SELinux</t>
+          <t>SELinux, archives, secure file transfer and tuning profiles</t>
         </is>
       </c>
       <c r="F32" s="22">
@@ -2390,7 +2390,7 @@
       <c r="J32" s="23" t="n"/>
       <c r="K32" s="21" t="inlineStr">
         <is>
-          <t>Hardest third of the module starts here. Weeks 9, 11 and 12 deserve the most revision time.</t>
+          <t>Hardest third of the module starts here. Weeks 10, 11 and 12 deserve the most revision time.</t>
         </is>
       </c>
     </row>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="E33" s="21" t="inlineStr">
         <is>
-          <t>Archives, secure file transfer and tuning profiles</t>
+          <t>SELinux, archives, secure file transfer and tuning profiles</t>
         </is>
       </c>
       <c r="F33" s="22">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="E34" s="21" t="inlineStr">
         <is>
-          <t>Archives, secure file transfer and tuning profiles</t>
+          <t>SELinux, archives, secure file transfer and tuning profiles</t>
         </is>
       </c>
       <c r="F34" s="22">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="E35" s="21" t="inlineStr">
         <is>
-          <t>Archives, secure file transfer and tuning profiles</t>
+          <t>SELinux, archives, secure file transfer and tuning profiles</t>
         </is>
       </c>
       <c r="F35" s="22">
@@ -3616,11 +3616,11 @@
       </c>
       <c r="C18" s="30" t="inlineStr">
         <is>
-          <t>week 9</t>
+          <t>week 10</t>
         </is>
       </c>
       <c r="D18" s="22">
-        <f>SemesterStart+7*(9-1)</f>
+        <f>SemesterStart+7*(10-1)</f>
         <v/>
       </c>
       <c r="E18" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Move RH134 chapter 12 from week 11 to week 12
Week 11 stopped before 12.01, so the chapter moves to week 12 in
full. The bootup(7) reading goes with it, and the planner weeks and
the study spreadsheet follow. Also corrects the planner's week for
practice challenge 13, left behind by the earlier 09.03 move.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planner/ict257-study-planner.xlsx
+++ b/planner/ict257-study-planner.xlsx
@@ -1045,7 +1045,7 @@
     <row r="39" ht="26" customHeight="1">
       <c r="A39" s="16" t="inlineStr">
         <is>
-          <t>ICT257 Red Hat System Administration, Singapore University of Social Sciences. Taught by Eugene Teo. Chapters and weeks follow lessons.md. Rebuild this file with python3 planner/build.py.</t>
+          <t>ICT257 Red Hat System Administration, Singapore University of Social Sciences. Taught by Eugene Teo. Chapters and weeks follow readings.md. Rebuild this file with python3 planner/build.py.</t>
         </is>
       </c>
     </row>
@@ -2539,7 +2539,7 @@
       </c>
       <c r="E36" s="21" t="inlineStr">
         <is>
-          <t>Partitions, swap, logical volumes and booting</t>
+          <t>Partitions, swap and logical volumes</t>
         </is>
       </c>
       <c r="F36" s="22">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="E37" s="21" t="inlineStr">
         <is>
-          <t>Partitions, swap, logical volumes and booting</t>
+          <t>Partitions, swap and logical volumes</t>
         </is>
       </c>
       <c r="F37" s="22">
@@ -2619,11 +2619,11 @@
         </is>
       </c>
       <c r="D38" s="19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E38" s="21" t="inlineStr">
         <is>
-          <t>Partitions, swap, logical volumes and booting</t>
+          <t>Booting, troubleshooting, firewalls and network file systems</t>
         </is>
       </c>
       <c r="F38" s="22">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="E39" s="21" t="inlineStr">
         <is>
-          <t>Boot troubleshooting, firewalls and network file systems</t>
+          <t>Booting, troubleshooting, firewalls and network file systems</t>
         </is>
       </c>
       <c r="F39" s="22">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E40" s="21" t="inlineStr">
         <is>
-          <t>Boot troubleshooting, firewalls and network file systems</t>
+          <t>Booting, troubleshooting, firewalls and network file systems</t>
         </is>
       </c>
       <c r="F40" s="22">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="E41" s="21" t="inlineStr">
         <is>
-          <t>Boot troubleshooting, firewalls and network file systems</t>
+          <t>Booting, troubleshooting, firewalls and network file systems</t>
         </is>
       </c>
       <c r="F41" s="22">
@@ -3576,11 +3576,11 @@
       </c>
       <c r="C17" s="30" t="inlineStr">
         <is>
-          <t>week 10</t>
+          <t>week 11</t>
         </is>
       </c>
       <c r="D17" s="22">
-        <f>SemesterStart+7*(10-1)</f>
+        <f>SemesterStart+7*(11-1)</f>
         <v/>
       </c>
       <c r="E17" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Move RH134 chapter 15 from week 12 to week 13
Week 12 stopped before 15.01, so the chapter moves to week 13 in
full. RHCSA-6.2 and 6.3 go with it, since only chapter 15 teaches
them, and review lab 19.03 now also waits for week 13. The planner
weeks and practice challenge 18 follow.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planner/ict257-study-planner.xlsx
+++ b/planner/ict257-study-planner.xlsx
@@ -1010,7 +1010,7 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>The two comprehensive reviews sit in week 14, where lessons.md puts them. RH124 20 is open to you from week 7 and RH134 19.02 to 19.04 from week 12, so start either one early if you can.</t>
+          <t>The two comprehensive reviews sit in week 14, where lessons.md puts them. RH124 20 is open to you from week 7 and RH134 19.02 and 19.04 from week 12, and 19.03 and 19.05 from week 13, so start either one early if you can.</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2390,7 @@
       <c r="J32" s="23" t="n"/>
       <c r="K32" s="21" t="inlineStr">
         <is>
-          <t>Hardest third of the module starts here. Weeks 10, 11 and 12 deserve the most revision time.</t>
+          <t>Hardest third of the module starts here. Weeks 10 to 13 deserve the most revision time.</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="E38" s="21" t="inlineStr">
         <is>
-          <t>Booting, troubleshooting, firewalls and network file systems</t>
+          <t>Booting, troubleshooting and firewalls</t>
         </is>
       </c>
       <c r="F38" s="22">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="E39" s="21" t="inlineStr">
         <is>
-          <t>Booting, troubleshooting, firewalls and network file systems</t>
+          <t>Booting, troubleshooting and firewalls</t>
         </is>
       </c>
       <c r="F39" s="22">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E40" s="21" t="inlineStr">
         <is>
-          <t>Booting, troubleshooting, firewalls and network file systems</t>
+          <t>Booting, troubleshooting and firewalls</t>
         </is>
       </c>
       <c r="F40" s="22">
@@ -2745,11 +2745,11 @@
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E41" s="21" t="inlineStr">
         <is>
-          <t>Booting, troubleshooting, firewalls and network file systems</t>
+          <t>Network file systems, installation, containers and image mode</t>
         </is>
       </c>
       <c r="F41" s="22">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="E42" s="21" t="inlineStr">
         <is>
-          <t>Installation, containers and image mode</t>
+          <t>Network file systems, installation, containers and image mode</t>
         </is>
       </c>
       <c r="F42" s="22">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="E43" s="21" t="inlineStr">
         <is>
-          <t>Installation, containers and image mode</t>
+          <t>Network file systems, installation, containers and image mode</t>
         </is>
       </c>
       <c r="F43" s="22">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="E44" s="21" t="inlineStr">
         <is>
-          <t>Installation, containers and image mode</t>
+          <t>Network file systems, installation, containers and image mode</t>
         </is>
       </c>
       <c r="F44" s="22">
@@ -2952,7 +2952,7 @@
       <c r="J45" s="23" t="n"/>
       <c r="K45" s="21" t="inlineStr">
         <is>
-          <t>Labs 19.02 to 19.04 are open from week 12. Lab 19.05 rests on week 13 containers.</t>
+          <t>Labs 19.02 and 19.04 are open from week 12. Labs 19.03 and 19.05 rest on week 13 material.</t>
         </is>
       </c>
     </row>
@@ -3776,11 +3776,11 @@
       </c>
       <c r="C22" s="30" t="inlineStr">
         <is>
-          <t>week 12</t>
+          <t>week 13</t>
         </is>
       </c>
       <c r="D22" s="22">
-        <f>SemesterStart+7*(12-1)</f>
+        <f>SemesterStart+7*(13-1)</f>
         <v/>
       </c>
       <c r="E22" s="19" t="inlineStr">

</xml_diff>